<commit_message>
Clarify which sheet needs two people.
Co-authored-by: Harsh Kharwar <harsh.240103263@iiitbh.ac.in>
</commit_message>
<xml_diff>
--- a/docs/TechZephyr-test-cases.xlsx
+++ b/docs/TechZephyr-test-cases.xlsx
@@ -697,7 +697,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Amber rows and the Two people sheet need Person A and Person B at the same time. White rows are one person.</t>
+          <t>The Two people sheet is entirely for paired testing. On Test cases, People is 1. On Accounts, the first three rows are the people who publish or review.</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3105,7 @@
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LTechZephyr CIT  ·  test cases&amp;CFilter People = 2 for the paired cases</oddHeader>
+    <oddHeader>&amp;LTechZephyr CIT  ·  test cases&amp;COne person per row. Paired flows are on the Two people sheet.</oddHeader>
     <oddFooter>&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>